<commit_message>
EC Final: Air China through tickets; record through-ticket checks
- EC Final Fly: Air China through tickets UB-HGH (CNY 3,265) and HGH-UB
  (CNY 2,250); the CNY 700 domestic assumption is not on sale for 25 Jan
- EC Final Train: return via through ticket, home 29 Jan, no Beijing night
- Nanjing/Shenyang plans: notes on through tickets checked (all dearer)
- Fares sheet: EC Final domestic + through-ticket rows; details.md updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ICPC_2026_Nanjing_Shenyang_Budget (2).xlsx
+++ b/ICPC_2026_Nanjing_Shenyang_Budget (2).xlsx
@@ -178,7 +178,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -400,6 +400,9 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -655,7 +658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="37" min="1" max="1"/>
@@ -1004,6 +1007,18 @@
       <c r="D23" s="51" t="inlineStr">
         <is>
           <t>Less class missed, sleep at home; ~4 extra travel legs; over ₮15M</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="75" t="inlineStr">
+        <is>
+          <t>Through tickets (checked 1 Oct)</t>
+        </is>
+      </c>
+      <c r="B25" s="74" t="inlineStr">
+        <is>
+          <t>Single Air China tickets UB → Nanjing ($353), Nanjing → UB ($360–394) and Shenyang → UB ($286) all cost more than MIAT + high-speed rail, so all three variants keep separate tickets.</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1188,7 @@
       </c>
       <c r="I15" s="63" t="inlineStr">
         <is>
-          <t>Trip.com 1 Oct: MIAT 17:15–19:30 $150 pp (SlickTrip 30 Sep: $154)</t>
+          <t>Trip.com 1 Oct: MIAT 17:15–19:30 $150 pp (SlickTrip 30 Sep: $154). Through tickets UB → Nanjing on 6 Nov cost more: Air China via Beijing $353, Spring/China Eastern via Shanghai $208 (no bag, lands 23:55)</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1393,7 @@
       </c>
       <c r="I21" s="63" t="inlineStr">
         <is>
-          <t>12306 fare 339 CNY</t>
+          <t>12306 fare 339 CNY Through ticket Shenyang 09:00 → Beijing → UB 15:05 (Air China, 16 Nov) is $286 pp on Trip.com 1 Oct – ~$50 pp dearer than train + Beijing night + Air China, but worth it if the closing ceremony runs late.</t>
         </is>
       </c>
     </row>
@@ -2195,7 +2210,7 @@
       </c>
       <c r="I15" s="63" t="inlineStr">
         <is>
-          <t>Trip.com 1 Oct: MIAT 17:15–19:30 $150 pp (SlickTrip 30 Sep: $154)</t>
+          <t>Trip.com 1 Oct: MIAT 17:15–19:30 $150 pp (SlickTrip 30 Sep: $154). Through tickets UB → Nanjing on 6 Nov cost more: Air China via Beijing $353, Spring/China Eastern via Shanghai $208 (no bag, lands 23:55)</t>
         </is>
       </c>
     </row>
@@ -2400,7 +2415,7 @@
       </c>
       <c r="I21" s="63" t="inlineStr">
         <is>
-          <t>12306 fare 339 CNY</t>
+          <t>12306 fare 339 CNY Through ticket Shenyang 09:00 → Beijing → UB 15:05 (Air China, 16 Nov) is $286 pp on Trip.com 1 Oct – ~$50 pp dearer than train + Beijing night + Air China, but worth it if the closing ceremony runs late.</t>
         </is>
       </c>
     </row>
@@ -3217,7 +3232,7 @@
       </c>
       <c r="I15" s="63" t="inlineStr">
         <is>
-          <t>Trip.com 1 Oct: MIAT 17:15–19:30 $150 pp (SlickTrip 30 Sep: $154)</t>
+          <t>Trip.com 1 Oct: MIAT 17:15–19:30 $150 pp (SlickTrip 30 Sep: $154). Through tickets UB → Nanjing on 6 Nov cost more: Air China via Beijing $353, Spring/China Eastern via Shanghai $208 (no bag, lands 23:55)</t>
         </is>
       </c>
     </row>
@@ -3255,7 +3270,7 @@
       </c>
       <c r="I16" s="63" t="inlineStr">
         <is>
-          <t>Trip.com 1 Oct: MIAT 20:45–23:05 $219 pp (SlickTrip $223). Air China 08:10 is $172 but needs an extra Beijing night on 9 Nov</t>
+          <t>Trip.com 1 Oct: MIAT 20:45–23:05 $219 pp (SlickTrip $223). Air China 08:10 is $172 but needs an extra Beijing night on 9 Nov. Nanjing → UB in one ticket on 10 Nov costs more: $360–394 via Beijing (vs fast train $75 + MIAT $219)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
New sources: Ctrip sleeper trains, Trip.com hotels, Hohhot route for EC Fly
- Shenyang plans: K53/K54 overnight sleepers replace G-trains + Beijing hotel nights
- Hotels near each venue re-priced on Trip.com (RiCH, Mujiangnan, Pod Inn, HanTing, Mehood Theater)
- EC Final Fly: Aero Mongolia UB->Hohhot + Xiamen Airlines Hohhot->Hangzhou (¥2,752 vs ¥3,265); 4-person total now under ₮15M
- Fares log: Hohhot rows and a "Trains & hotels" sheet; details.md records the sources and URL patterns

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ICPC_2026_Nanjing_Shenyang_Budget (2).xlsx
+++ b/ICPC_2026_Nanjing_Shenyang_Budget (2).xlsx
@@ -658,7 +658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="37" min="1" max="1"/>
@@ -675,7 +675,7 @@
     <row r="2" ht="15" customHeight="1" s="38">
       <c r="A2" s="40" t="inlineStr">
         <is>
-          <t>3 contestants from Ulaanbaatar. Prices checked 30 Sep 2026; flights re-priced on Trip.com 30 Sep – 1 Oct 2026. Blue = inputs; yellow = key assumptions; green = links to another sheet.</t>
+          <t>3 contestants from Ulaanbaatar. Prices checked 30 Sep 2026; flights re-priced on Trip.com 30 Sep – 1 Oct 2026; trains (Ctrip) and hotels (Trip.com) re-checked 1 Oct. Blue = inputs; yellow = key assumptions; green = links to another sheet.</t>
         </is>
       </c>
     </row>
@@ -930,17 +930,17 @@
       </c>
       <c r="B20" s="51" t="inlineStr">
         <is>
-          <t>~500 m walk</t>
+          <t>~1 km walk</t>
         </is>
       </c>
       <c r="C20" s="51" t="inlineStr">
         <is>
-          <t>~50–60 min metro</t>
+          <t>~15 min metro</t>
         </is>
       </c>
       <c r="D20" s="51" t="inlineStr">
         <is>
-          <t>~500 m walk</t>
+          <t>~1 km walk</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="B21" s="51" t="inlineStr">
         <is>
-          <t>~1.4 km</t>
+          <t>~1.3 km</t>
         </is>
       </c>
       <c r="C21" s="51" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="D21" s="51" t="inlineStr">
         <is>
-          <t>~1.4 km</t>
+          <t>~1.3 km</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="B23" s="51" t="inlineStr">
         <is>
-          <t>Best rest &amp; least commuting on contest days; ~₮2.3M headroom</t>
+          <t>Best rest &amp; least commuting on contest days; ~₮2.8M headroom</t>
         </is>
       </c>
       <c r="C23" s="51" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="D23" s="51" t="inlineStr">
         <is>
-          <t>Less class missed, sleep at home; ~4 extra travel legs; over ₮15M</t>
+          <t>Less class missed, sleep at home; ~4 extra travel legs; subtotal fits ₮15M but ~₮0.6M over once the 10% contingency is added</t>
         </is>
       </c>
     </row>
@@ -1019,6 +1019,18 @@
       <c r="B25" s="74" t="inlineStr">
         <is>
           <t>Single Air China tickets UB → Nanjing ($353), Nanjing → UB ($360–394) and Shenyang → UB ($286) all cost more than MIAT + high-speed rail, so all three variants keep separate tickets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="75" t="inlineStr">
+        <is>
+          <t>New sources (checked 1 Oct)</t>
+        </is>
+      </c>
+      <c r="B26" s="74" t="inlineStr">
+        <is>
+          <t>Ctrip train timetables: overnight K53/K54 sleepers Beijing ⇄ Shenyang (¥171 hard / ¥263 soft) replace a G-train + Beijing hotel night. Trip.com hotels near each venue (family rooms) undercut Booking.com.</t>
         </is>
       </c>
     </row>
@@ -1363,16 +1375,16 @@
       <c r="A21" s="56" t="n"/>
       <c r="B21" s="57" t="inlineStr">
         <is>
-          <t>High-speed rail Shenyang North → Beijing Chaoyang, 2nd class (~2 h 45 min)</t>
+          <t>Overnight train K54 Shenyang North 22:00 → Beijing 06:58, soft sleeper</t>
         </is>
       </c>
       <c r="C21" s="57" t="inlineStr">
         <is>
-          <t>15 Nov (eve)</t>
+          <t>15 Nov (night)</t>
         </is>
       </c>
       <c r="D21" s="58" t="n">
-        <v>339</v>
+        <v>263</v>
       </c>
       <c r="E21" s="59" t="inlineStr">
         <is>
@@ -1393,7 +1405,7 @@
       </c>
       <c r="I21" s="63" t="inlineStr">
         <is>
-          <t>12306 fare 339 CNY Through ticket Shenyang 09:00 → Beijing → UB 15:05 (Air China, 16 Nov) is $286 pp on Trip.com 1 Oct – ~$50 pp dearer than train + Beijing night + Air China, but worth it if the closing ceremony runs late.</t>
+          <t>Ctrip 1 Oct: K54 hard sleeper ¥171, soft sleeper ¥263 (4-berth cabin). Leaves 22:00, so a late closing ceremony is fine; replaces the evening G-train (¥339) + a Beijing hotel night. Air China through ticket SHE 09:00 → UB 15:05 ($286) is the fallback. Sales open 15 days ahead (31 Oct).</t>
         </is>
       </c>
     </row>
@@ -1453,7 +1465,7 @@
       <c r="A24" s="56" t="n"/>
       <c r="B24" s="57" t="inlineStr">
         <is>
-          <t>Magnotel NUAA Shengtai West Road (~500 m walk to NUAA Jiangjun Rd campus)</t>
+          <t>Mujiangnan Hotel, Cuipingshan (~1 km walk to NUAA Jiangjun Rd campus), Smart Family Room</t>
         </is>
       </c>
       <c r="C24" s="57" t="inlineStr">
@@ -1462,7 +1474,7 @@
         </is>
       </c>
       <c r="D24" s="58" t="n">
-        <v>602.67</v>
+        <v>251.33</v>
       </c>
       <c r="E24" s="59" t="inlineStr">
         <is>
@@ -1482,7 +1494,7 @@
       </c>
       <c r="I24" s="63" t="inlineStr">
         <is>
-          <t>Booking.com 7–13 Nov, 3 adults/1 room: 3,616 CNY for 6 nights = 602.67/night</t>
+          <t>Trip.com 1 Oct: ¥1,508 for 6 nights (3 adults, 1 room); rated 9.2 (1,355 reviews). Was Magnotel ¥602.67/night</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1502,7 @@
       <c r="A25" s="56" t="n"/>
       <c r="B25" s="57" t="inlineStr">
         <is>
-          <t>Atour Hotel Shenyang Youth Street Golden Gallery (~1.4 km to NEU Nanhu campus)</t>
+          <t>Shenyang RiCH Hotel, Sanhao St (~1.3 km to NEU Nanhu; Family Room sleeps 4)</t>
         </is>
       </c>
       <c r="C25" s="57" t="inlineStr">
@@ -1499,7 +1511,7 @@
         </is>
       </c>
       <c r="D25" s="58" t="n">
-        <v>524</v>
+        <v>338</v>
       </c>
       <c r="E25" s="59" t="inlineStr">
         <is>
@@ -1519,46 +1531,20 @@
       </c>
       <c r="I25" s="63" t="inlineStr">
         <is>
-          <t>Booking.com 13–15 Nov, 3 adults/1 room: 1,048 CNY for 2 nights, rated 9.5</t>
+          <t>Trip.com 1 Oct: ¥676 for 2 nights (3 adults); rated 9.6 (1,802 reviews). Was Atour ¥524/night</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="38">
       <c r="A26" s="56" t="n"/>
-      <c r="B26" s="57" t="inlineStr">
-        <is>
-          <t>Beijing budget hotel near Chaoyang station / airport</t>
-        </is>
-      </c>
-      <c r="C26" s="57" t="inlineStr">
-        <is>
-          <t>15 Nov (1 night)</t>
-        </is>
-      </c>
-      <c r="D26" s="58" t="n">
-        <v>300</v>
-      </c>
-      <c r="E26" s="59" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="F26" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="G26" s="61">
-        <f>D26*F26</f>
-        <v/>
-      </c>
-      <c r="H26" s="62">
-        <f>G26*IF(E26="USD",Compare!$B$7,IF(E26="CNY",Compare!$B$8,1))</f>
-        <v/>
-      </c>
-      <c r="I26" s="63" t="inlineStr">
-        <is>
-          <t>Same rate as 6 Nov Beijing search</t>
-        </is>
-      </c>
+      <c r="B26" s="57" t="n"/>
+      <c r="C26" s="57" t="n"/>
+      <c r="D26" s="58" t="n"/>
+      <c r="E26" s="59" t="n"/>
+      <c r="F26" s="64" t="n"/>
+      <c r="G26" s="61" t="n"/>
+      <c r="H26" s="62" t="n"/>
+      <c r="I26" s="63" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="38">
       <c r="A27" s="54" t="inlineStr">
@@ -2385,16 +2371,16 @@
       <c r="A21" s="56" t="n"/>
       <c r="B21" s="57" t="inlineStr">
         <is>
-          <t>High-speed rail Shenyang North → Beijing Chaoyang, 2nd class (~2 h 45 min)</t>
+          <t>Overnight train K54 Shenyang North 22:00 → Beijing 06:58, hard sleeper</t>
         </is>
       </c>
       <c r="C21" s="57" t="inlineStr">
         <is>
-          <t>15 Nov (eve)</t>
+          <t>15 Nov (night)</t>
         </is>
       </c>
       <c r="D21" s="58" t="n">
-        <v>339</v>
+        <v>171</v>
       </c>
       <c r="E21" s="59" t="inlineStr">
         <is>
@@ -2415,7 +2401,7 @@
       </c>
       <c r="I21" s="63" t="inlineStr">
         <is>
-          <t>12306 fare 339 CNY Through ticket Shenyang 09:00 → Beijing → UB 15:05 (Air China, 16 Nov) is $286 pp on Trip.com 1 Oct – ~$50 pp dearer than train + Beijing night + Air China, but worth it if the closing ceremony runs late.</t>
+          <t>Ctrip 1 Oct: K54 hard sleeper ¥171, soft sleeper ¥263 (4-berth cabin). Leaves 22:00, so a late closing ceremony is fine; replaces the evening G-train (¥339) + a Beijing hotel night. Air China through ticket SHE 09:00 → UB 15:05 ($286) is the fallback. Sales open 15 days ahead (31 Oct).</t>
         </is>
       </c>
     </row>
@@ -2475,7 +2461,7 @@
       <c r="A24" s="56" t="n"/>
       <c r="B24" s="57" t="inlineStr">
         <is>
-          <t>Jinjiang Inn Nanjing Train Station 1 (Gulou; ~50–60 min metro to NUAA Jiangjun Rd)</t>
+          <t>Pod Inn Nanjing South Station North Plaza (~3.8 km to NUAA, ~15 min metro), Family Room</t>
         </is>
       </c>
       <c r="C24" s="57" t="inlineStr">
@@ -2484,7 +2470,7 @@
         </is>
       </c>
       <c r="D24" s="58" t="n">
-        <v>145</v>
+        <v>109.67</v>
       </c>
       <c r="E24" s="59" t="inlineStr">
         <is>
@@ -2504,7 +2490,7 @@
       </c>
       <c r="I24" s="63" t="inlineStr">
         <is>
-          <t>Booking.com: 725 CNY for 5 nights (7–12 Nov) = 145/night; rated 7.1</t>
+          <t>Trip.com 1 Oct: ¥658 for 6 nights (3 adults, 1 room); rated 8.4 (2,374 reviews). Was Jinjiang Inn Nanjing Station ¥145/night, ~50–60 min metro</t>
         </is>
       </c>
     </row>
@@ -2541,46 +2527,20 @@
       </c>
       <c r="I25" s="63" t="inlineStr">
         <is>
-          <t>Booking.com: 258 CNY for 3 nights = 86/night. Unusually cheap – re-check</t>
+          <t>Booking.com: 258 CNY for 3 nights = 86/night. Trip.com 1 Oct: rated 8.2 from 1,062 reviews – the low price is real</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="38">
       <c r="A26" s="56" t="n"/>
-      <c r="B26" s="57" t="inlineStr">
-        <is>
-          <t>Beijing hostel near Chaoyang station</t>
-        </is>
-      </c>
-      <c r="C26" s="57" t="inlineStr">
-        <is>
-          <t>15 Nov (1 night)</t>
-        </is>
-      </c>
-      <c r="D26" s="58" t="n">
-        <v>227</v>
-      </c>
-      <c r="E26" s="59" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="F26" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="G26" s="61">
-        <f>D26*F26</f>
-        <v/>
-      </c>
-      <c r="H26" s="62">
-        <f>G26*IF(E26="USD",Compare!$B$7,IF(E26="CNY",Compare!$B$8,1))</f>
-        <v/>
-      </c>
-      <c r="I26" s="63" t="inlineStr">
-        <is>
-          <t>Same rate as 6 Nov hostel</t>
-        </is>
-      </c>
+      <c r="B26" s="57" t="n"/>
+      <c r="C26" s="57" t="n"/>
+      <c r="D26" s="58" t="n"/>
+      <c r="E26" s="59" t="n"/>
+      <c r="F26" s="64" t="n"/>
+      <c r="G26" s="61" t="n"/>
+      <c r="H26" s="62" t="n"/>
+      <c r="I26" s="63" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="38">
       <c r="A27" s="54" t="inlineStr">
@@ -3445,16 +3405,16 @@
       <c r="A22" s="56" t="n"/>
       <c r="B22" s="57" t="inlineStr">
         <is>
-          <t>High-speed rail Beijing Chaoyang → Shenyang North (~2 h 45 min)</t>
+          <t>Overnight train K53 Beijing 22:35 → Shenyang North 07:00, soft sleeper</t>
         </is>
       </c>
       <c r="C22" s="57" t="inlineStr">
         <is>
-          <t>14 Nov (morning)</t>
+          <t>13 Nov (night)</t>
         </is>
       </c>
       <c r="D22" s="58" t="n">
-        <v>339</v>
+        <v>263</v>
       </c>
       <c r="E22" s="59" t="inlineStr">
         <is>
@@ -3475,7 +3435,7 @@
       </c>
       <c r="I22" s="63" t="inlineStr">
         <is>
-          <t>12306 fare 339 CNY</t>
+          <t>Ctrip 1 Oct: K53 soft sleeper ¥263 (hard ¥171). Replaces the Beijing night + morning G-train (¥339). MIAT lands 19:30, so ~1 h 20 min spare after immigration + Airport Express; if MIAT is late, change the ticket (1 free change) to the 14 Nov G-train. Sales open 15 days ahead (29 Oct).</t>
         </is>
       </c>
     </row>
@@ -3483,16 +3443,16 @@
       <c r="A23" s="56" t="n"/>
       <c r="B23" s="57" t="inlineStr">
         <is>
-          <t>High-speed rail Shenyang North → Beijing Chaoyang, 2nd class (~2 h 45 min)</t>
+          <t>Overnight train K54 Shenyang North 22:00 → Beijing 06:58, soft sleeper</t>
         </is>
       </c>
       <c r="C23" s="57" t="inlineStr">
         <is>
-          <t>15 Nov (eve)</t>
+          <t>15 Nov (night)</t>
         </is>
       </c>
       <c r="D23" s="58" t="n">
-        <v>339</v>
+        <v>263</v>
       </c>
       <c r="E23" s="59" t="inlineStr">
         <is>
@@ -3513,7 +3473,7 @@
       </c>
       <c r="I23" s="63" t="inlineStr">
         <is>
-          <t>12306 fare 339 CNY</t>
+          <t>Ctrip 1 Oct: K54 hard sleeper ¥171, soft sleeper ¥263 (4-berth cabin). Leaves 22:00, so a late closing ceremony is fine; replaces the evening G-train (¥339) + a Beijing hotel night. Air China through ticket SHE 09:00 → UB 15:05 ($286) is the fallback. Sales open 15 days ahead (31 Oct).</t>
         </is>
       </c>
     </row>
@@ -3573,7 +3533,7 @@
       <c r="A26" s="56" t="n"/>
       <c r="B26" s="57" t="inlineStr">
         <is>
-          <t>Magnotel NUAA Shengtai West Road (~500 m walk to NUAA Jiangjun Rd campus)</t>
+          <t>Mujiangnan Hotel, Cuipingshan (~1 km walk to NUAA Jiangjun Rd campus), Smart Family Room</t>
         </is>
       </c>
       <c r="C26" s="57" t="inlineStr">
@@ -3582,7 +3542,7 @@
         </is>
       </c>
       <c r="D26" s="58" t="n">
-        <v>602.67</v>
+        <v>250.67</v>
       </c>
       <c r="E26" s="59" t="inlineStr">
         <is>
@@ -3602,52 +3562,26 @@
       </c>
       <c r="I26" s="63" t="inlineStr">
         <is>
-          <t>Booking.com 7–13 Nov, 3 adults/1 room: 3,616 CNY for 6 nights = 602.67/night (rate assumed to hold for 3 nights)</t>
+          <t>Trip.com 1 Oct: ¥752 for 3 nights (3 adults, 1 room); rated 9.2 (1,355 reviews). Was Magnotel ¥602.67/night</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="38">
       <c r="A27" s="56" t="n"/>
-      <c r="B27" s="57" t="inlineStr">
-        <is>
-          <t>Beijing budget hotel near Chaoyang station</t>
-        </is>
-      </c>
-      <c r="C27" s="57" t="inlineStr">
-        <is>
-          <t>13 Nov (1 night)</t>
-        </is>
-      </c>
-      <c r="D27" s="65" t="n">
-        <v>300</v>
-      </c>
-      <c r="E27" s="59" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="F27" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="G27" s="61">
-        <f>D27*F27</f>
-        <v/>
-      </c>
-      <c r="H27" s="62">
-        <f>G27*IF(E27="USD",Compare!$B$7,IF(E27="CNY",Compare!$B$8,1))</f>
-        <v/>
-      </c>
-      <c r="I27" s="63" t="inlineStr">
-        <is>
-          <t>ASSUMPTION same Beijing rate</t>
-        </is>
-      </c>
+      <c r="B27" s="57" t="n"/>
+      <c r="C27" s="57" t="n"/>
+      <c r="D27" s="65" t="n"/>
+      <c r="E27" s="59" t="n"/>
+      <c r="F27" s="64" t="n"/>
+      <c r="G27" s="61" t="n"/>
+      <c r="H27" s="62" t="n"/>
+      <c r="I27" s="63" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1" s="38">
       <c r="A28" s="56" t="n"/>
       <c r="B28" s="57" t="inlineStr">
         <is>
-          <t>Atour Hotel Shenyang Youth Street Golden Gallery (~1.4 km to NEU Nanhu campus)</t>
+          <t>Shenyang RiCH Hotel, Sanhao St (~1.3 km to NEU Nanhu; Family Room sleeps 4)</t>
         </is>
       </c>
       <c r="C28" s="57" t="inlineStr">
@@ -3656,7 +3590,7 @@
         </is>
       </c>
       <c r="D28" s="58" t="n">
-        <v>524</v>
+        <v>338</v>
       </c>
       <c r="E28" s="59" t="inlineStr">
         <is>
@@ -3676,46 +3610,20 @@
       </c>
       <c r="I28" s="63" t="inlineStr">
         <is>
-          <t>Booking.com 13–15 Nov, 3 adults/1 room: 1,048 CNY for 2 nights, rated 9.5 (rate assumed for 1 night)</t>
+          <t>Trip.com 1 Oct: ¥338 for 1 night (3 adults); rated 9.6 (1,802 reviews). Was Atour ¥524</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="38">
       <c r="A29" s="56" t="n"/>
-      <c r="B29" s="57" t="inlineStr">
-        <is>
-          <t>Beijing budget hotel near Chaoyang station / airport</t>
-        </is>
-      </c>
-      <c r="C29" s="57" t="inlineStr">
-        <is>
-          <t>15 Nov (1 night)</t>
-        </is>
-      </c>
-      <c r="D29" s="58" t="n">
-        <v>300</v>
-      </c>
-      <c r="E29" s="59" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="F29" s="64" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" s="61">
-        <f>D29*F29</f>
-        <v/>
-      </c>
-      <c r="H29" s="62">
-        <f>G29*IF(E29="USD",Compare!$B$7,IF(E29="CNY",Compare!$B$8,1))</f>
-        <v/>
-      </c>
-      <c r="I29" s="63" t="inlineStr">
-        <is>
-          <t>Same Beijing rate</t>
-        </is>
-      </c>
+      <c r="B29" s="57" t="n"/>
+      <c r="C29" s="57" t="n"/>
+      <c r="D29" s="58" t="n"/>
+      <c r="E29" s="59" t="n"/>
+      <c r="F29" s="64" t="n"/>
+      <c r="G29" s="61" t="n"/>
+      <c r="H29" s="62" t="n"/>
+      <c r="I29" s="63" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1" s="38">
       <c r="A30" s="54" t="inlineStr">
@@ -4276,7 +4184,7 @@
       </c>
       <c r="C4" s="74" t="inlineStr">
         <is>
-          <t>Morning G-train Beijing South → Nanjing South (A: ~3 h 25 min fast train; B: ~4 h 50 min). Check-in &amp; practice at NUAA Jiangjun Road campus.</t>
+          <t>Morning G-train Beijing South → Nanjing South (A: ~3 h 25 min fast train; B: ~4 h 50 min). Check-in &amp; practice at NUAA Jiangjun Road campus. A: Mujiangnan Hotel (~1 km walk); B: Pod Inn (~15 min metro).</t>
         </is>
       </c>
     </row>
@@ -4327,7 +4235,7 @@
       </c>
       <c r="C7" s="74" t="inlineStr">
         <is>
-          <t>China Eastern Nanjing 07:40 → Shenyang 09:50 (bag included). Free afternoon to rest; hotel near NEU.</t>
+          <t>China Eastern Nanjing 07:40 → Shenyang 09:50 (bag included). Free afternoon to rest; A: RiCH Hotel near NEU; B: Bestay.</t>
         </is>
       </c>
     </row>
@@ -4356,12 +4264,12 @@
       </c>
       <c r="B9" s="74" t="inlineStr">
         <is>
-          <t>Beijing</t>
+          <t>Train</t>
         </is>
       </c>
       <c r="C9" s="74" t="inlineStr">
         <is>
-          <t>SHENYANG REGIONAL contest day. Evening G-train Shenyang North → Beijing Chaoyang (~2 h 45 min).</t>
+          <t>SHENYANG REGIONAL contest day. K54 overnight sleeper Shenyang North 22:00 → Beijing 06:58 (A: soft, B: hard sleeper).</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4286,7 @@
       </c>
       <c r="C10" s="74" t="inlineStr">
         <is>
-          <t>Air China Beijing Capital 12:55 → UB 15:05 (nonstop).</t>
+          <t>Beijing station → PEK by metro + Airport Express. Air China Beijing Capital 12:55 → UB 15:05 (nonstop).</t>
         </is>
       </c>
     </row>
@@ -4516,12 +4424,12 @@
       </c>
       <c r="B20" s="74" t="inlineStr">
         <is>
-          <t>Beijing</t>
+          <t>Train</t>
         </is>
       </c>
       <c r="C20" s="74" t="inlineStr">
         <is>
-          <t>MIAT OM223 UB 17:15 → Beijing 19:30. Hotel near Beijing Chaoyang station.</t>
+          <t>MIAT OM223 UB 17:15 → Beijing 19:30. Airport Express + metro to Beijing station; K53 soft sleeper 22:35 → Shenyang North 07:00.</t>
         </is>
       </c>
     </row>
@@ -4538,7 +4446,7 @@
       </c>
       <c r="C21" s="74" t="inlineStr">
         <is>
-          <t>Morning G-train Beijing Chaoyang → Shenyang North (~2 h 45 min). Check-in &amp; practice at NEU Nanhu.</t>
+          <t>Arrive Shenyang 07:00, RiCH Hotel near NEU. Check-in &amp; practice at NEU Nanhu.</t>
         </is>
       </c>
     </row>
@@ -4550,12 +4458,12 @@
       </c>
       <c r="B22" s="74" t="inlineStr">
         <is>
-          <t>Beijing</t>
+          <t>Train</t>
         </is>
       </c>
       <c r="C22" s="74" t="inlineStr">
         <is>
-          <t>SHENYANG REGIONAL contest day. Evening train back to Beijing.</t>
+          <t>SHENYANG REGIONAL contest day. K54 soft sleeper Shenyang North 22:00 → Beijing 06:58.</t>
         </is>
       </c>
     </row>
@@ -4572,7 +4480,7 @@
       </c>
       <c r="C23" s="74" t="inlineStr">
         <is>
-          <t>Air China Beijing Capital 12:55 → UB 15:05 (nonstop).</t>
+          <t>Beijing station → PEK by metro + Airport Express. Air China Beijing Capital 12:55 → UB 15:05 (nonstop).</t>
         </is>
       </c>
     </row>
@@ -4596,7 +4504,7 @@
       </c>
       <c r="C26" s="74" t="inlineStr">
         <is>
-          <t>If the Shenyang awards ceremony runs late on 15 Nov: sleep in Shenyang, train on 16 Nov, fly MIAT OM224 17 Nov 20:45 (same fare) – roughly +1 Beijing night.</t>
+          <t>The K54 sleeper leaves Shenyang North at 22:00, so a late awards ceremony on 15 Nov is fine. If it runs past ~21:15, take the Air China through ticket SHE 09:00 → UB 15:05 on 16 Nov ($286 pp) and sleep in Shenyang.</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4516,7 @@
       </c>
       <c r="C27" s="74" t="inlineStr">
         <is>
-          <t>Chinese train tickets open ~15 days before travel on 12306 / Trip.com; passports needed to buy.</t>
+          <t>Chinese train tickets open 15 days before travel on 12306 / Trip.com / Ctrip; passports needed to buy. Beijing → Nanjing sleepers (D5 21:21) leave too soon after MIAT lands at 19:30, so the 6 Nov Beijing night stays.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
12306 + ChinaTicketOnline: overnight sleepers for EC Final and Nanjing → Shenyang
- EC Final Train: D17 Beijing 19:10 → Hangzhou 09:15 sleeper (¥491) replaces the
  G-train + 25 Jan hotel night; fix the double-counted Hangzhou East taxi
- Combined A/B: Z366 Nanjing → Shenyang North sleeper replaces China Eastern $121
  + the 12 Nov Nanjing night
- Official 12306 fares and station sale times; correct sale dates (D − 14 days)
- New "12306 & ChinaTicketOnline" sheet: reseller is 30–70% dearer, not used
- details.md: 12306 and ChinaTicketOnline query recipes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ICPC_2026_Nanjing_Shenyang_Budget (2).xlsx
+++ b/ICPC_2026_Nanjing_Shenyang_Budget (2).xlsx
@@ -658,7 +658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="37" min="1" max="1"/>
@@ -675,10 +675,11 @@
     <row r="2" ht="15" customHeight="1" s="38">
       <c r="A2" s="40" t="inlineStr">
         <is>
-          <t>3 contestants from Ulaanbaatar. Prices checked 30 Sep 2026; flights re-priced on Trip.com 30 Sep – 1 Oct 2026; trains (Ctrip) and hotels (Trip.com) re-checked 1 Oct. Blue = inputs; yellow = key assumptions; green = links to another sheet.</t>
-        </is>
-      </c>
-    </row>
+          <t>3 contestants from Ulaanbaatar. Prices checked 30 Sep 2026; flights re-priced on Trip.com 30 Sep – 1 Oct 2026; trains (Ctrip) and hotels (Trip.com) re-checked 1 Oct; official fares and sale times from 12306 on 3 Oct. Blue = inputs; yellow = key assumptions; green = links to another sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="38">
       <c r="A4" s="41" t="inlineStr">
         <is>
@@ -761,6 +762,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="38">
       <c r="A11" s="41" t="inlineStr">
         <is>
@@ -996,7 +998,7 @@
       </c>
       <c r="B23" s="51" t="inlineStr">
         <is>
-          <t>Best rest &amp; least commuting on contest days; ~₮2.8M headroom</t>
+          <t>Best rest &amp; least commuting on contest days; ~₮3.4M headroom</t>
         </is>
       </c>
       <c r="C23" s="51" t="inlineStr">
@@ -1010,6 +1012,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="75" t="inlineStr">
         <is>
@@ -1031,6 +1034,18 @@
       <c r="B26" s="74" t="inlineStr">
         <is>
           <t>Ctrip train timetables: overnight K53/K54 sleepers Beijing ⇄ Shenyang (¥171 hard / ¥263 soft) replace a G-train + Beijing hotel night. Trip.com hotels near each venue (family rooms) undercut Booking.com.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="75" t="inlineStr">
+        <is>
+          <t>12306 (checked 3 Oct)</t>
+        </is>
+      </c>
+      <c r="B27" s="74" t="inlineStr">
+        <is>
+          <t>A and B: the Z366 overnight sleeper Nanjing 16:58 → Shenyang North 09:14 (hard ¥337 / soft ¥530) replaces the China Eastern flight ($121) and the 12 Nov Nanjing hotel night. ChinaTicketOnline resells the same trains at ~30–70% more once its $8.50–20 per-ticket fee is added – not used.</t>
         </is>
       </c>
     </row>
@@ -1075,6 +1090,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="38">
       <c r="A4" s="41" t="inlineStr">
         <is>
@@ -1104,6 +1120,12 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13" ht="30" customHeight="1" s="38">
       <c r="A13" s="53" t="inlineStr">
         <is>
@@ -1208,16 +1230,16 @@
       <c r="A16" s="56" t="n"/>
       <c r="B16" s="57" t="inlineStr">
         <is>
-          <t>China Eastern Nanjing → Shenyang, nonstop 07:40–09:50 (checked bag included)</t>
+          <t>Air China Beijing (PEK) → Ulaanbaatar, nonstop 12:55–15:05</t>
         </is>
       </c>
       <c r="C16" s="57" t="inlineStr">
         <is>
-          <t>13 Nov</t>
+          <t>16 Nov</t>
         </is>
       </c>
       <c r="D16" s="58" t="n">
-        <v>121</v>
+        <v>171</v>
       </c>
       <c r="E16" s="59" t="inlineStr">
         <is>
@@ -1238,66 +1260,43 @@
       </c>
       <c r="I16" s="63" t="inlineStr">
         <is>
-          <t>Trip.com 1 Oct: $121 pp incl. bag. Replaces Spring 9C7758 19:55–23:50 ($110.67 + ~100 CNY bag = ~$125.6). Backup: Shenzhen Airlines 19:25–21:30 $129</t>
+          <t>Trip.com 30 Sep: Air China nonstop $171 pp (MIAT OM224 11:30 was $194 on Trip.com, $196.33 on SlickTrip)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="38">
-      <c r="A17" s="56" t="n"/>
-      <c r="B17" s="57" t="inlineStr">
-        <is>
-          <t>Checked bag – included in the China Eastern fare</t>
-        </is>
-      </c>
-      <c r="C17" s="57" t="inlineStr">
-        <is>
-          <t>13 Nov</t>
-        </is>
-      </c>
-      <c r="D17" s="58" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="59" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="F17" s="60">
-        <f>Compare!$B$6</f>
-        <v/>
-      </c>
-      <c r="G17" s="61">
-        <f>D17*F17</f>
-        <v/>
-      </c>
-      <c r="H17" s="62">
-        <f>G17*IF(E17="USD",Compare!$B$7,IF(E17="CNY",Compare!$B$8,1))</f>
-        <v/>
-      </c>
-      <c r="I17" s="63" t="inlineStr">
-        <is>
-          <t>Was ~100 CNY/bag on Spring Airlines; not needed now</t>
-        </is>
-      </c>
+      <c r="A17" s="54" t="inlineStr">
+        <is>
+          <t>Trains</t>
+        </is>
+      </c>
+      <c r="B17" s="55" t="n"/>
+      <c r="C17" s="55" t="n"/>
+      <c r="D17" s="55" t="n"/>
+      <c r="E17" s="55" t="n"/>
+      <c r="F17" s="55" t="n"/>
+      <c r="G17" s="55" t="n"/>
+      <c r="H17" s="55" t="n"/>
+      <c r="I17" s="55" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="38">
       <c r="A18" s="56" t="n"/>
       <c r="B18" s="57" t="inlineStr">
         <is>
-          <t>Air China Beijing (PEK) → Ulaanbaatar, nonstop 12:55–15:05</t>
+          <t>High-speed rail Beijing South → Nanjing South, fast G-train (~3 h 25 min)</t>
         </is>
       </c>
       <c r="C18" s="57" t="inlineStr">
         <is>
-          <t>16 Nov</t>
+          <t>7 Nov</t>
         </is>
       </c>
       <c r="D18" s="58" t="n">
-        <v>171</v>
+        <v>504</v>
       </c>
       <c r="E18" s="59" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CNY</t>
         </is>
       </c>
       <c r="F18" s="60">
@@ -1314,39 +1313,62 @@
       </c>
       <c r="I18" s="63" t="inlineStr">
         <is>
-          <t>Trip.com 30 Sep: Air China nonstop $171 pp (MIAT OM224 11:30 was $194 on Trip.com, $196.33 on SlickTrip)</t>
+          <t>Ctrip: 504 CNY on the ~3 h 23 min trains (slower ~4 h 50 min trains are 445)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="38">
-      <c r="A19" s="54" t="inlineStr">
-        <is>
-          <t>Trains</t>
-        </is>
-      </c>
-      <c r="B19" s="55" t="n"/>
-      <c r="C19" s="55" t="n"/>
-      <c r="D19" s="55" t="n"/>
-      <c r="E19" s="55" t="n"/>
-      <c r="F19" s="55" t="n"/>
-      <c r="G19" s="55" t="n"/>
-      <c r="H19" s="55" t="n"/>
-      <c r="I19" s="55" t="n"/>
+      <c r="A19" s="56" t="n"/>
+      <c r="B19" s="57" t="inlineStr">
+        <is>
+          <t>Overnight train Z366 Nanjing 16:58 → Shenyang North 09:14 (+1), soft sleeper (4-berth cabin)</t>
+        </is>
+      </c>
+      <c r="C19" s="57" t="inlineStr">
+        <is>
+          <t>12 Nov (night)</t>
+        </is>
+      </c>
+      <c r="D19" s="58" t="n">
+        <v>530</v>
+      </c>
+      <c r="E19" s="59" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="F19" s="60">
+        <f>Compare!$B$6</f>
+        <v/>
+      </c>
+      <c r="G19" s="61">
+        <f>D19*F19</f>
+        <v/>
+      </c>
+      <c r="H19" s="62">
+        <f>G19*IF(E19="USD",Compare!$B$7,IF(E19="CNY",Compare!$B$8,1))</f>
+        <v/>
+      </c>
+      <c r="I19" s="63" t="inlineStr">
+        <is>
+          <t>12306 3 Oct (official fare, 15 Oct train): Z366 hard sleeper ¥337, soft ¥530. Replaces China Eastern 13 Nov 07:40 ($121) + the 12 Nov Nanjing hotel night, and lands at the same time. Sales open 29 Oct 08:15 (Nanjing station). Backups: Z516 18:38 → 10:26, Z176 18:32 → 10:42 (same fares); the China Eastern flight.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="38">
       <c r="A20" s="56" t="n"/>
       <c r="B20" s="57" t="inlineStr">
         <is>
-          <t>High-speed rail Beijing South → Nanjing South, fast G-train (~3 h 25 min)</t>
+          <t>Overnight train K54 Shenyang North 22:00 → Beijing 06:58, soft sleeper</t>
         </is>
       </c>
       <c r="C20" s="57" t="inlineStr">
         <is>
-          <t>7 Nov</t>
+          <t>15 Nov (night)</t>
         </is>
       </c>
       <c r="D20" s="58" t="n">
-        <v>504</v>
+        <v>263</v>
       </c>
       <c r="E20" s="59" t="inlineStr">
         <is>
@@ -1367,47 +1389,20 @@
       </c>
       <c r="I20" s="63" t="inlineStr">
         <is>
-          <t>Ctrip: 504 CNY on the ~3 h 23 min trains (slower ~4 h 50 min trains are 445)</t>
+          <t>Ctrip 1 Oct: K54 hard sleeper ¥171, soft sleeper ¥263 (4-berth cabin). Leaves 22:00, so a late closing ceremony is fine; replaces the evening G-train (¥339) + a Beijing hotel night. Air China through ticket SHE 09:00 → UB 15:05 ($286) is the fallback. 12306 3 Oct: same official fares; sales open 1 Nov 09:00 (Shenyang North).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="38">
       <c r="A21" s="56" t="n"/>
-      <c r="B21" s="57" t="inlineStr">
-        <is>
-          <t>Overnight train K54 Shenyang North 22:00 → Beijing 06:58, soft sleeper</t>
-        </is>
-      </c>
-      <c r="C21" s="57" t="inlineStr">
-        <is>
-          <t>15 Nov (night)</t>
-        </is>
-      </c>
-      <c r="D21" s="58" t="n">
-        <v>263</v>
-      </c>
-      <c r="E21" s="59" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="F21" s="60">
-        <f>Compare!$B$6</f>
-        <v/>
-      </c>
-      <c r="G21" s="61">
-        <f>D21*F21</f>
-        <v/>
-      </c>
-      <c r="H21" s="62">
-        <f>G21*IF(E21="USD",Compare!$B$7,IF(E21="CNY",Compare!$B$8,1))</f>
-        <v/>
-      </c>
-      <c r="I21" s="63" t="inlineStr">
-        <is>
-          <t>Ctrip 1 Oct: K54 hard sleeper ¥171, soft sleeper ¥263 (4-berth cabin). Leaves 22:00, so a late closing ceremony is fine; replaces the evening G-train (¥339) + a Beijing hotel night. Air China through ticket SHE 09:00 → UB 15:05 ($286) is the fallback. Sales open 15 days ahead (31 Oct).</t>
-        </is>
-      </c>
+      <c r="B21" s="57" t="n"/>
+      <c r="C21" s="57" t="n"/>
+      <c r="D21" s="58" t="n"/>
+      <c r="E21" s="59" t="n"/>
+      <c r="F21" s="64" t="n"/>
+      <c r="G21" s="61" t="n"/>
+      <c r="H21" s="62" t="n"/>
+      <c r="I21" s="63" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="38">
       <c r="A22" s="54" t="inlineStr">
@@ -1470,7 +1465,7 @@
       </c>
       <c r="C24" s="57" t="inlineStr">
         <is>
-          <t>7–13 Nov (6 nights)</t>
+          <t>7–12 Nov (5 nights)</t>
         </is>
       </c>
       <c r="D24" s="58" t="n">
@@ -1482,7 +1477,7 @@
         </is>
       </c>
       <c r="F24" s="64" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G24" s="61">
         <f>D24*F24</f>
@@ -1494,7 +1489,7 @@
       </c>
       <c r="I24" s="63" t="inlineStr">
         <is>
-          <t>Trip.com 1 Oct: ¥1,508 for 6 nights (3 adults, 1 room); rated 9.2 (1,355 reviews). Was Magnotel ¥602.67/night</t>
+          <t>Trip.com 1 Oct: ¥1,508 for 6 nights (3 adults, 1 room); rated 9.2 (1,355 reviews). Was Magnotel ¥602.67/night. Plan books 5 of these nights; 12 Nov is on the Z366 sleeper.</t>
         </is>
       </c>
     </row>
@@ -1880,6 +1875,7 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
     <row r="39" ht="15" customHeight="1" s="38">
       <c r="G39" s="66" t="inlineStr">
         <is>
@@ -1913,6 +1909,7 @@
         <v/>
       </c>
     </row>
+    <row r="42"/>
     <row r="43" ht="15" customHeight="1" s="38">
       <c r="G43" s="57" t="inlineStr">
         <is>
@@ -1957,6 +1954,7 @@
         <v/>
       </c>
     </row>
+    <row r="47"/>
     <row r="48" ht="15" customHeight="1" s="38">
       <c r="G48" s="41" t="inlineStr">
         <is>
@@ -2071,6 +2069,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="38">
       <c r="A4" s="41" t="inlineStr">
         <is>
@@ -2100,6 +2099,12 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13" ht="30" customHeight="1" s="38">
       <c r="A13" s="53" t="inlineStr">
         <is>
@@ -2204,16 +2209,16 @@
       <c r="A16" s="56" t="n"/>
       <c r="B16" s="57" t="inlineStr">
         <is>
-          <t>China Eastern Nanjing → Shenyang, nonstop 07:40–09:50 (checked bag included)</t>
+          <t>Air China Beijing (PEK) → Ulaanbaatar, nonstop 12:55–15:05</t>
         </is>
       </c>
       <c r="C16" s="57" t="inlineStr">
         <is>
-          <t>13 Nov</t>
+          <t>16 Nov</t>
         </is>
       </c>
       <c r="D16" s="58" t="n">
-        <v>121</v>
+        <v>171</v>
       </c>
       <c r="E16" s="59" t="inlineStr">
         <is>
@@ -2234,66 +2239,43 @@
       </c>
       <c r="I16" s="63" t="inlineStr">
         <is>
-          <t>Trip.com 1 Oct: $121 pp incl. bag. Replaces Spring 9C7758 19:55–23:50 ($110.67 + ~100 CNY bag = ~$125.6). Backup: Shenzhen Airlines 19:25–21:30 $129</t>
+          <t>Trip.com 30 Sep: Air China nonstop $171 pp (MIAT OM224 11:30 was $194 on Trip.com, $196.33 on SlickTrip)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="38">
-      <c r="A17" s="56" t="n"/>
-      <c r="B17" s="57" t="inlineStr">
-        <is>
-          <t>Checked bag – included in the China Eastern fare</t>
-        </is>
-      </c>
-      <c r="C17" s="57" t="inlineStr">
-        <is>
-          <t>13 Nov</t>
-        </is>
-      </c>
-      <c r="D17" s="58" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="59" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="F17" s="60">
-        <f>Compare!$B$6</f>
-        <v/>
-      </c>
-      <c r="G17" s="61">
-        <f>D17*F17</f>
-        <v/>
-      </c>
-      <c r="H17" s="62">
-        <f>G17*IF(E17="USD",Compare!$B$7,IF(E17="CNY",Compare!$B$8,1))</f>
-        <v/>
-      </c>
-      <c r="I17" s="63" t="inlineStr">
-        <is>
-          <t>Was ~100 CNY/bag on Spring Airlines; not needed now</t>
-        </is>
-      </c>
+      <c r="A17" s="54" t="inlineStr">
+        <is>
+          <t>Trains</t>
+        </is>
+      </c>
+      <c r="B17" s="55" t="n"/>
+      <c r="C17" s="55" t="n"/>
+      <c r="D17" s="55" t="n"/>
+      <c r="E17" s="55" t="n"/>
+      <c r="F17" s="55" t="n"/>
+      <c r="G17" s="55" t="n"/>
+      <c r="H17" s="55" t="n"/>
+      <c r="I17" s="55" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="38">
       <c r="A18" s="56" t="n"/>
       <c r="B18" s="57" t="inlineStr">
         <is>
-          <t>Air China Beijing (PEK) → Ulaanbaatar, nonstop 12:55–15:05</t>
+          <t>High-speed rail Beijing South → Nanjing South, slower G-train (~4 h 35–50 min)</t>
         </is>
       </c>
       <c r="C18" s="57" t="inlineStr">
         <is>
-          <t>16 Nov</t>
+          <t>7 Nov</t>
         </is>
       </c>
       <c r="D18" s="58" t="n">
-        <v>171</v>
+        <v>445</v>
       </c>
       <c r="E18" s="59" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CNY</t>
         </is>
       </c>
       <c r="F18" s="60">
@@ -2310,39 +2292,62 @@
       </c>
       <c r="I18" s="63" t="inlineStr">
         <is>
-          <t>Trip.com 30 Sep: Air China nonstop $171 pp (MIAT OM224 11:30 was $194 on Trip.com, $196.33 on SlickTrip)</t>
+          <t>Ctrip: 445 CNY 2nd class</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="38">
-      <c r="A19" s="54" t="inlineStr">
-        <is>
-          <t>Trains</t>
-        </is>
-      </c>
-      <c r="B19" s="55" t="n"/>
-      <c r="C19" s="55" t="n"/>
-      <c r="D19" s="55" t="n"/>
-      <c r="E19" s="55" t="n"/>
-      <c r="F19" s="55" t="n"/>
-      <c r="G19" s="55" t="n"/>
-      <c r="H19" s="55" t="n"/>
-      <c r="I19" s="55" t="n"/>
+      <c r="A19" s="56" t="n"/>
+      <c r="B19" s="57" t="inlineStr">
+        <is>
+          <t>Overnight train Z366 Nanjing 16:58 → Shenyang North 09:14 (+1), hard sleeper</t>
+        </is>
+      </c>
+      <c r="C19" s="57" t="inlineStr">
+        <is>
+          <t>12 Nov (night)</t>
+        </is>
+      </c>
+      <c r="D19" s="58" t="n">
+        <v>337</v>
+      </c>
+      <c r="E19" s="59" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="F19" s="60">
+        <f>Compare!$B$6</f>
+        <v/>
+      </c>
+      <c r="G19" s="61">
+        <f>D19*F19</f>
+        <v/>
+      </c>
+      <c r="H19" s="62">
+        <f>G19*IF(E19="USD",Compare!$B$7,IF(E19="CNY",Compare!$B$8,1))</f>
+        <v/>
+      </c>
+      <c r="I19" s="63" t="inlineStr">
+        <is>
+          <t>12306 3 Oct (official fare, 15 Oct train): Z366 hard sleeper ¥337, soft ¥530. Replaces China Eastern 13 Nov 07:40 ($121) + the 12 Nov Nanjing hotel night, and lands at the same time. Sales open 29 Oct 08:15 (Nanjing station). Backups: Z516 18:38 → 10:26, Z176 18:32 → 10:42 (same fares); the China Eastern flight.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="38">
       <c r="A20" s="56" t="n"/>
       <c r="B20" s="57" t="inlineStr">
         <is>
-          <t>High-speed rail Beijing South → Nanjing South, slower G-train (~4 h 35–50 min)</t>
+          <t>Overnight train K54 Shenyang North 22:00 → Beijing 06:58, hard sleeper</t>
         </is>
       </c>
       <c r="C20" s="57" t="inlineStr">
         <is>
-          <t>7 Nov</t>
+          <t>15 Nov (night)</t>
         </is>
       </c>
       <c r="D20" s="58" t="n">
-        <v>445</v>
+        <v>171</v>
       </c>
       <c r="E20" s="59" t="inlineStr">
         <is>
@@ -2363,47 +2368,20 @@
       </c>
       <c r="I20" s="63" t="inlineStr">
         <is>
-          <t>Ctrip: 445 CNY 2nd class</t>
+          <t>Ctrip 1 Oct: K54 hard sleeper ¥171, soft sleeper ¥263 (4-berth cabin). Leaves 22:00, so a late closing ceremony is fine; replaces the evening G-train (¥339) + a Beijing hotel night. Air China through ticket SHE 09:00 → UB 15:05 ($286) is the fallback. 12306 3 Oct: same official fares; sales open 1 Nov 09:00 (Shenyang North).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="38">
       <c r="A21" s="56" t="n"/>
-      <c r="B21" s="57" t="inlineStr">
-        <is>
-          <t>Overnight train K54 Shenyang North 22:00 → Beijing 06:58, hard sleeper</t>
-        </is>
-      </c>
-      <c r="C21" s="57" t="inlineStr">
-        <is>
-          <t>15 Nov (night)</t>
-        </is>
-      </c>
-      <c r="D21" s="58" t="n">
-        <v>171</v>
-      </c>
-      <c r="E21" s="59" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="F21" s="60">
-        <f>Compare!$B$6</f>
-        <v/>
-      </c>
-      <c r="G21" s="61">
-        <f>D21*F21</f>
-        <v/>
-      </c>
-      <c r="H21" s="62">
-        <f>G21*IF(E21="USD",Compare!$B$7,IF(E21="CNY",Compare!$B$8,1))</f>
-        <v/>
-      </c>
-      <c r="I21" s="63" t="inlineStr">
-        <is>
-          <t>Ctrip 1 Oct: K54 hard sleeper ¥171, soft sleeper ¥263 (4-berth cabin). Leaves 22:00, so a late closing ceremony is fine; replaces the evening G-train (¥339) + a Beijing hotel night. Air China through ticket SHE 09:00 → UB 15:05 ($286) is the fallback. Sales open 15 days ahead (31 Oct).</t>
-        </is>
-      </c>
+      <c r="B21" s="57" t="n"/>
+      <c r="C21" s="57" t="n"/>
+      <c r="D21" s="58" t="n"/>
+      <c r="E21" s="59" t="n"/>
+      <c r="F21" s="64" t="n"/>
+      <c r="G21" s="61" t="n"/>
+      <c r="H21" s="62" t="n"/>
+      <c r="I21" s="63" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="38">
       <c r="A22" s="54" t="inlineStr">
@@ -2466,7 +2444,7 @@
       </c>
       <c r="C24" s="57" t="inlineStr">
         <is>
-          <t>7–13 Nov (6 nights)</t>
+          <t>7–12 Nov (5 nights)</t>
         </is>
       </c>
       <c r="D24" s="58" t="n">
@@ -2478,7 +2456,7 @@
         </is>
       </c>
       <c r="F24" s="64" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G24" s="61">
         <f>D24*F24</f>
@@ -2490,7 +2468,7 @@
       </c>
       <c r="I24" s="63" t="inlineStr">
         <is>
-          <t>Trip.com 1 Oct: ¥658 for 6 nights (3 adults, 1 room); rated 8.4 (2,374 reviews). Was Jinjiang Inn Nanjing Station ¥145/night, ~50–60 min metro</t>
+          <t>Trip.com 1 Oct: ¥658 for 6 nights (3 adults, 1 room); rated 8.4 (2,374 reviews). Was Jinjiang Inn Nanjing Station ¥145/night, ~50–60 min metro Plan books 5 of these nights; 12 Nov is on the Z366 sleeper.</t>
         </is>
       </c>
     </row>
@@ -2876,6 +2854,7 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
     <row r="39" ht="15" customHeight="1" s="38">
       <c r="G39" s="66" t="inlineStr">
         <is>
@@ -2909,6 +2888,7 @@
         <v/>
       </c>
     </row>
+    <row r="42"/>
     <row r="43" ht="15" customHeight="1" s="38">
       <c r="G43" s="57" t="inlineStr">
         <is>
@@ -2953,6 +2933,7 @@
         <v/>
       </c>
     </row>
+    <row r="47"/>
     <row r="48" ht="15" customHeight="1" s="38">
       <c r="G48" s="41" t="inlineStr">
         <is>
@@ -3067,6 +3048,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="38">
       <c r="A4" s="41" t="inlineStr">
         <is>
@@ -3096,6 +3078,12 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13" ht="30" customHeight="1" s="38">
       <c r="A13" s="53" t="inlineStr">
         <is>
@@ -3435,7 +3423,7 @@
       </c>
       <c r="I22" s="63" t="inlineStr">
         <is>
-          <t>Ctrip 1 Oct: K53 soft sleeper ¥263 (hard ¥171). Replaces the Beijing night + morning G-train (¥339). MIAT lands 19:30, so ~1 h 20 min spare after immigration + Airport Express; if MIAT is late, change the ticket (1 free change) to the 14 Nov G-train. Sales open 15 days ahead (29 Oct).</t>
+          <t>Ctrip 1 Oct: K53 soft sleeper ¥263 (hard ¥171). Replaces the Beijing night + morning G-train (¥339). MIAT lands 19:30, so ~1 h 20 min spare after immigration + Airport Express; if MIAT is late, change the ticket (1 free change) to the 14 Nov G-train. 12306 3 Oct: same official fares; sales open 30 Oct 10:00 (Beijing station). Backup if K53 is sold out: K341 Beijing 23:00 → Shenyang 08:47, hard sleeper ¥194.</t>
         </is>
       </c>
     </row>
@@ -3473,7 +3461,7 @@
       </c>
       <c r="I23" s="63" t="inlineStr">
         <is>
-          <t>Ctrip 1 Oct: K54 hard sleeper ¥171, soft sleeper ¥263 (4-berth cabin). Leaves 22:00, so a late closing ceremony is fine; replaces the evening G-train (¥339) + a Beijing hotel night. Air China through ticket SHE 09:00 → UB 15:05 ($286) is the fallback. Sales open 15 days ahead (31 Oct).</t>
+          <t>Ctrip 1 Oct: K54 hard sleeper ¥171, soft sleeper ¥263 (4-berth cabin). Leaves 22:00, so a late closing ceremony is fine; replaces the evening G-train (¥339) + a Beijing hotel night. Air China through ticket SHE 09:00 → UB 15:05 ($286) is the fallback. 12306 3 Oct: same official fares; sales open 1 Nov 09:00 (Shenyang North).</t>
         </is>
       </c>
     </row>
@@ -3959,6 +3947,7 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42" ht="15" customHeight="1" s="38">
       <c r="G42" s="66" t="inlineStr">
         <is>
@@ -3992,6 +3981,7 @@
         <v/>
       </c>
     </row>
+    <row r="45"/>
     <row r="46" ht="15" customHeight="1" s="38">
       <c r="G46" s="57" t="inlineStr">
         <is>
@@ -4036,6 +4026,7 @@
         <v/>
       </c>
     </row>
+    <row r="50"/>
     <row r="51" ht="15" customHeight="1" s="38">
       <c r="G51" s="41" t="inlineStr">
         <is>
@@ -4213,12 +4204,12 @@
       </c>
       <c r="B6" s="74" t="inlineStr">
         <is>
-          <t>Nanjing</t>
+          <t>Nanjing (12 Nov: train)</t>
         </is>
       </c>
       <c r="C6" s="74" t="inlineStr">
         <is>
-          <t>Rest / upsolve / train in Nanjing.</t>
+          <t>Rest / upsolve / train in Nanjing. 12 Nov: check out, Z366 overnight sleeper Nanjing 16:58 → Shenyang North 09:14 (A: soft, B: hard sleeper).</t>
         </is>
       </c>
     </row>
@@ -4235,7 +4226,7 @@
       </c>
       <c r="C7" s="74" t="inlineStr">
         <is>
-          <t>China Eastern Nanjing 07:40 → Shenyang 09:50 (bag included). Free afternoon to rest; A: RiCH Hotel near NEU; B: Bestay.</t>
+          <t>Arrive Shenyang North 09:14. Free day to rest; A: RiCH Hotel near NEU; B: Bestay.</t>
         </is>
       </c>
     </row>
@@ -4290,6 +4281,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="15" customHeight="1" s="38">
       <c r="A12" s="73" t="inlineStr">
         <is>
@@ -4484,6 +4476,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25" ht="26.85" customHeight="1" s="38">
       <c r="A25" s="41" t="inlineStr">
         <is>
@@ -4516,7 +4509,7 @@
       </c>
       <c r="C27" s="74" t="inlineStr">
         <is>
-          <t>Chinese train tickets open 15 days before travel on 12306 / Trip.com / Ctrip; passports needed to buy. Beijing → Nanjing sleepers (D5 21:21) leave too soon after MIAT lands at 19:30, so the 6 Nov Beijing night stays.</t>
+          <t>Chinese train tickets open 15 days before travel (day of travel counts, e.g. 13 Nov trains on 30 Oct) on 12306 / Trip.com / Ctrip; passports needed to buy. Beijing → Nanjing sleepers (D5 21:21) leave too soon after MIAT lands at 19:30, so the 6 Nov Beijing night stays.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plan around sleep: protect pre-contest nights, cheapest after
- New 'Sleep check' sheet with per-plan audit of the nights before each contest
- Pre-contest upgrades: Shenyang Budget K53 soft sleeper; new Hong Kong - Sleep first
- Post-contest downgrades: K54 hard sleeper, Shanghai D8 seat, Nanchang D136 seat
- Compare picks regenerated from computed totals; older workbook K54 hard sleeper
- details.md: sleep principle and updated results

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ICPC_2026_Nanjing_Shenyang_Budget (2).xlsx
+++ b/ICPC_2026_Nanjing_Shenyang_Budget (2).xlsx
@@ -679,7 +679,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="38">
       <c r="A4" s="41" t="inlineStr">
         <is>
@@ -762,7 +761,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="38">
       <c r="A11" s="41" t="inlineStr">
         <is>
@@ -998,7 +996,7 @@
       </c>
       <c r="B23" s="51" t="inlineStr">
         <is>
-          <t>Best rest &amp; least commuting on contest days; ~₮3.4M headroom</t>
+          <t>Best rest &amp; least commuting on contest days; ~₮3.6M headroom</t>
         </is>
       </c>
       <c r="C23" s="51" t="inlineStr">
@@ -1012,7 +1010,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="75" t="inlineStr">
         <is>
@@ -1090,7 +1087,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="38">
       <c r="A4" s="41" t="inlineStr">
         <is>
@@ -1120,12 +1116,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13" ht="30" customHeight="1" s="38">
       <c r="A13" s="53" t="inlineStr">
         <is>
@@ -1359,7 +1349,7 @@
       <c r="A20" s="56" t="n"/>
       <c r="B20" s="57" t="inlineStr">
         <is>
-          <t>Overnight train K54 Shenyang North 22:00 → Beijing 06:58, soft sleeper</t>
+          <t>Overnight train K54 Shenyang North 22:00 → Beijing 06:58, hard sleeper (after the contest)</t>
         </is>
       </c>
       <c r="C20" s="57" t="inlineStr">
@@ -1368,7 +1358,7 @@
         </is>
       </c>
       <c r="D20" s="58" t="n">
-        <v>263</v>
+        <v>171</v>
       </c>
       <c r="E20" s="59" t="inlineStr">
         <is>
@@ -1389,7 +1379,7 @@
       </c>
       <c r="I20" s="63" t="inlineStr">
         <is>
-          <t>Ctrip 1 Oct: K54 hard sleeper ¥171, soft sleeper ¥263 (4-berth cabin). Leaves 22:00, so a late closing ceremony is fine; replaces the evening G-train (¥339) + a Beijing hotel night. Air China through ticket SHE 09:00 → UB 15:05 ($286) is the fallback. 12306 3 Oct: same official fares; sales open 1 Nov 09:00 (Shenyang North).</t>
+          <t>Ctrip 1 Oct / 12306: K54 hard sleeper ¥171 (soft ¥263). Hard on purpose: after the contest sleep no longer matters. Leaves 22:00, so a late closing ceremony is fine; replaces the evening G-train (¥339) + a Beijing hotel night. Air China through ticket SHE 09:00 → UB 15:05 ($286) is the fallback. Sales open 1 Nov 09:00 (Shenyang North).</t>
         </is>
       </c>
     </row>
@@ -1875,7 +1865,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39" ht="15" customHeight="1" s="38">
       <c r="G39" s="66" t="inlineStr">
         <is>
@@ -1909,7 +1898,6 @@
         <v/>
       </c>
     </row>
-    <row r="42"/>
     <row r="43" ht="15" customHeight="1" s="38">
       <c r="G43" s="57" t="inlineStr">
         <is>
@@ -1954,7 +1942,6 @@
         <v/>
       </c>
     </row>
-    <row r="47"/>
     <row r="48" ht="15" customHeight="1" s="38">
       <c r="G48" s="41" t="inlineStr">
         <is>
@@ -2069,7 +2056,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="38">
       <c r="A4" s="41" t="inlineStr">
         <is>
@@ -2099,12 +2085,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13" ht="30" customHeight="1" s="38">
       <c r="A13" s="53" t="inlineStr">
         <is>
@@ -2854,7 +2834,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39" ht="15" customHeight="1" s="38">
       <c r="G39" s="66" t="inlineStr">
         <is>
@@ -2888,7 +2867,6 @@
         <v/>
       </c>
     </row>
-    <row r="42"/>
     <row r="43" ht="15" customHeight="1" s="38">
       <c r="G43" s="57" t="inlineStr">
         <is>
@@ -2933,7 +2911,6 @@
         <v/>
       </c>
     </row>
-    <row r="47"/>
     <row r="48" ht="15" customHeight="1" s="38">
       <c r="G48" s="41" t="inlineStr">
         <is>
@@ -3048,7 +3025,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="38">
       <c r="A4" s="41" t="inlineStr">
         <is>
@@ -3078,12 +3054,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13" ht="30" customHeight="1" s="38">
       <c r="A13" s="53" t="inlineStr">
         <is>
@@ -3431,7 +3401,7 @@
       <c r="A23" s="56" t="n"/>
       <c r="B23" s="57" t="inlineStr">
         <is>
-          <t>Overnight train K54 Shenyang North 22:00 → Beijing 06:58, soft sleeper</t>
+          <t>Overnight train K54 Shenyang North 22:00 → Beijing 06:58, hard sleeper (after the contest)</t>
         </is>
       </c>
       <c r="C23" s="57" t="inlineStr">
@@ -3440,7 +3410,7 @@
         </is>
       </c>
       <c r="D23" s="58" t="n">
-        <v>263</v>
+        <v>171</v>
       </c>
       <c r="E23" s="59" t="inlineStr">
         <is>
@@ -3461,7 +3431,7 @@
       </c>
       <c r="I23" s="63" t="inlineStr">
         <is>
-          <t>Ctrip 1 Oct: K54 hard sleeper ¥171, soft sleeper ¥263 (4-berth cabin). Leaves 22:00, so a late closing ceremony is fine; replaces the evening G-train (¥339) + a Beijing hotel night. Air China through ticket SHE 09:00 → UB 15:05 ($286) is the fallback. 12306 3 Oct: same official fares; sales open 1 Nov 09:00 (Shenyang North).</t>
+          <t>Ctrip 1 Oct / 12306: K54 hard sleeper ¥171 (soft ¥263). Hard on purpose: after the contest sleep no longer matters. Leaves 22:00, so a late closing ceremony is fine; replaces the evening G-train (¥339) + a Beijing hotel night. Air China through ticket SHE 09:00 → UB 15:05 ($286) is the fallback. Sales open 1 Nov 09:00 (Shenyang North).</t>
         </is>
       </c>
     </row>
@@ -3947,7 +3917,6 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42" ht="15" customHeight="1" s="38">
       <c r="G42" s="66" t="inlineStr">
         <is>
@@ -3981,7 +3950,6 @@
         <v/>
       </c>
     </row>
-    <row r="45"/>
     <row r="46" ht="15" customHeight="1" s="38">
       <c r="G46" s="57" t="inlineStr">
         <is>
@@ -4026,7 +3994,6 @@
         <v/>
       </c>
     </row>
-    <row r="50"/>
     <row r="51" ht="15" customHeight="1" s="38">
       <c r="G51" s="41" t="inlineStr">
         <is>
@@ -4209,7 +4176,7 @@
       </c>
       <c r="C6" s="74" t="inlineStr">
         <is>
-          <t>Rest / upsolve / train in Nanjing. 12 Nov: check out, Z366 overnight sleeper Nanjing 16:58 → Shenyang North 09:14 (A: soft, B: hard sleeper).</t>
+          <t>Rest / upsolve / train in Nanjing. 12 Nov: check out, Z366 overnight sleeper Nanjing 16:58 → Shenyang North 09:14 (hard sleeper; after the contest).</t>
         </is>
       </c>
     </row>
@@ -4260,7 +4227,7 @@
       </c>
       <c r="C9" s="74" t="inlineStr">
         <is>
-          <t>SHENYANG REGIONAL contest day. K54 overnight sleeper Shenyang North 22:00 → Beijing 06:58 (A: soft, B: hard sleeper).</t>
+          <t>SHENYANG REGIONAL contest day. K54 overnight sleeper Shenyang North 22:00 → Beijing 06:58 (hard sleeper; after the contest).</t>
         </is>
       </c>
     </row>
@@ -4281,7 +4248,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="15" customHeight="1" s="38">
       <c r="A12" s="73" t="inlineStr">
         <is>
@@ -4455,7 +4421,7 @@
       </c>
       <c r="C22" s="74" t="inlineStr">
         <is>
-          <t>SHENYANG REGIONAL contest day. K54 soft sleeper Shenyang North 22:00 → Beijing 06:58.</t>
+          <t>SHENYANG REGIONAL contest day. K54 hard sleeper Shenyang North 22:00 → Beijing 06:58.</t>
         </is>
       </c>
     </row>
@@ -4476,7 +4442,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25" ht="26.85" customHeight="1" s="38">
       <c r="A25" s="41" t="inlineStr">
         <is>

</xml_diff>